<commit_message>
Add free contractor estimate template page + xlsx, estimate tab in toolkit, sitewide Open Graph and breadcrumb schema
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xkz1HZBUbxbmBDh3iB1XeW
</commit_message>
<xml_diff>
--- a/docs/distribution/product/contractor-pricing-toolkit.xlsx
+++ b/docs/distribution/product/contractor-pricing-toolkit.xlsx
@@ -12,8 +12,11 @@
     <sheet name="Hourly Rate" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Change Order" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Job Profit Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Customer Estimate" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Customer Estimate'!$A$1:$E$40</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -24,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,6 +100,32 @@
       <color rgb="00FF6A2B"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF6A2B"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00586273"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F1B2D"/>
+    </font>
+    <font>
+      <color rgb="00586273"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="009AA6BA"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -143,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +204,23 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -540,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -612,45 +658,55 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>6. Customer Estimate: a clean estimate to send the customer, with line items, tax, deposit and signature line.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Margin = profit ÷ price.  Markup = profit ÷ cost.  A 30% margin needs a 42.9% markup.</t>
-        </is>
-      </c>
+      <c r="A11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>Margin = profit ÷ price.  Markup = profit ÷ cost.  A 30% margin needs a 42.9% markup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>Google Sheets: File &gt; Import &gt; Upload this file. Excel: just open it.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>The numbers already filled in are examples. Replace them with your own.</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Figures are planning estimates only. This workbook is not accounting, tax or legal advice.</t>
+          <t>The numbers already filled in are examples. Replace them with your own.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>Figures are planning estimates only. This workbook is not accounting, tax or legal advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>Questions: hello@cleverloopdigital.com</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2094,4 +2150,448 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>[Your Business Name]</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="29" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>[Address] · [Phone] · [Email] · License # [000000]</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Prepared for</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Estimate #</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>[Customer name]</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>[Job address]</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Valid until</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>[Phone / email]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Job description</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>[Describe the work in one or two sentences]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>Item / description</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>Unit price</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="E14" s="24">
+        <f>IF(OR(B14="",D14=""),"",B14*D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Materials (see list)</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E15" s="24">
+        <f>IF(OR(B15="",D15=""),"",B15*D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Equipment rental</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>150</v>
+      </c>
+      <c r="E16" s="24">
+        <f>IF(OR(B16="",D16=""),"",B16*D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Disposal / dump fee</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>load</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" s="24">
+        <f>IF(OR(B17="",D17=""),"",B17*D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="n"/>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="24">
+        <f>IF(OR(B18="",D18=""),"",B18*D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="24">
+        <f>IF(OR(B19="",D19=""),"",B19*D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="24">
+        <f>IF(OR(B20="",D20=""),"",B20*D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="24">
+        <f>IF(OR(B21="",D21=""),"",B21*D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="24">
+        <f>IF(OR(B22="",D22=""),"",B22*D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="24">
+        <f>IF(OR(B23="",D23=""),"",B23*D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="24">
+        <f>IF(OR(B24="",D24=""),"",B24*D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="24">
+        <f>IF(OR(B25="",D25=""),"",B25*D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="E27" s="35">
+        <f>SUM(E14:E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Taxable amount (e.g. materials) $</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>Sales tax</t>
+        </is>
+      </c>
+      <c r="E28" s="35">
+        <f>B28*B29/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sales tax rate %</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E29" s="37">
+        <f>E27+E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Deposit %</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>Deposit due to start</t>
+        </is>
+      </c>
+      <c r="E30" s="35">
+        <f>E29*B30/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="D31" s="34" t="inlineStr">
+        <is>
+          <t>Balance on completion</t>
+        </is>
+      </c>
+      <c r="E31" s="35">
+        <f>E29-E30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>[Edit to match your business and your state's rules.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>Price valid until the date above. Work not listed here is extra and needs a signed change order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>Deposit due on acceptance; balance due on completion. [Accepted payment methods.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Accepted by (customer signature): ______________________     Date: __________</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="39" t="inlineStr">
+        <is>
+          <t>Template by Clever Loop Digital · cleverloopdigital.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add free contractor invoice template page + xlsx, invoice tab in paid toolkit, sitewide invoice links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xkz1HWVBPgsYwp1Xwsur6b
</commit_message>
<xml_diff>
--- a/docs/distribution/product/contractor-pricing-toolkit.xlsx
+++ b/docs/distribution/product/contractor-pricing-toolkit.xlsx
@@ -13,9 +13,11 @@
     <sheet name="Change Order" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Job Profit Log" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Customer Estimate" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Customer Invoice" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Customer Estimate'!$A$1:$E$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Customer Invoice'!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,48 +667,52 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>7. Customer Invoice: bill the finished job, subtract the deposit and show the balance due.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Margin = profit ÷ price.  Markup = profit ÷ cost.  A 30% margin needs a 42.9% markup.</t>
-        </is>
-      </c>
+      <c r="A12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>Margin = profit ÷ price.  Markup = profit ÷ cost.  A 30% margin needs a 42.9% markup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>Google Sheets: File &gt; Import &gt; Upload this file. Excel: just open it.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n"/>
-    </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>The numbers already filled in are examples. Replace them with your own.</t>
-        </is>
-      </c>
+      <c r="A15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Figures are planning estimates only. This workbook is not accounting, tax or legal advice.</t>
+          <t>The numbers already filled in are examples. Replace them with your own.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Figures are planning estimates only. This workbook is not accounting, tax or legal advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>Questions: hello@cleverloopdigital.com</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2594,4 +2600,482 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>[Your Business Name]</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="29" t="inlineStr">
+        <is>
+          <t>INVOICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>[Address] · [Phone] · [Email] · License # [000000]</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bill to</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Invoice #</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>[Customer name]</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Invoice date</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>[Job address]</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Due date</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>[Phone / email]</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Estimate #</t>
+        </is>
+      </c>
+      <c r="E8" s="31" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Work completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>[Describe the finished work and the completion date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>Item / description</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>Unit price</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="E14" s="24">
+        <f>IF(OR(B14="",D14=""),"",B14*D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Materials (see list)</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E15" s="24">
+        <f>IF(OR(B15="",D15=""),"",B15*D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Equipment rental</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>150</v>
+      </c>
+      <c r="E16" s="24">
+        <f>IF(OR(B16="",D16=""),"",B16*D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Disposal / dump fee</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>load</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" s="24">
+        <f>IF(OR(B17="",D17=""),"",B17*D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Change order #1 (signed)</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="n">
+        <v>822</v>
+      </c>
+      <c r="E18" s="24">
+        <f>IF(OR(B18="",D18=""),"",B18*D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="24">
+        <f>IF(OR(B19="",D19=""),"",B19*D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="24">
+        <f>IF(OR(B20="",D20=""),"",B20*D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="24">
+        <f>IF(OR(B21="",D21=""),"",B21*D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="24">
+        <f>IF(OR(B22="",D22=""),"",B22*D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="24">
+        <f>IF(OR(B23="",D23=""),"",B23*D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="24">
+        <f>IF(OR(B24="",D24=""),"",B24*D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="24">
+        <f>IF(OR(B25="",D25=""),"",B25*D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="E27" s="35">
+        <f>SUM(E14:E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Taxable amount (e.g. materials) $</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>Sales tax</t>
+        </is>
+      </c>
+      <c r="E28" s="35">
+        <f>B28*B29/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sales tax rate %</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>Invoice total</t>
+        </is>
+      </c>
+      <c r="E29" s="35">
+        <f>E27+E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Deposit already received $</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="n">
+        <v>793.5</v>
+      </c>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>Less deposit received</t>
+        </is>
+      </c>
+      <c r="E30" s="35">
+        <f>-B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Other payments received $</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="34" t="inlineStr">
+        <is>
+          <t>Less other payments</t>
+        </is>
+      </c>
+      <c r="E31" s="35">
+        <f>-B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>BALANCE DUE</t>
+        </is>
+      </c>
+      <c r="E32" s="37">
+        <f>E29+E30+E31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>[How to pay: check payable to ..., bank transfer, card link. Edit to match your business.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>Payment due by the due date above. [Late fee policy, if any, as allowed by your state and your contract.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>Thank you for your business.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>Template by Clever Loop Digital · cleverloopdigital.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>